<commit_message>
Rebuild LCI matrix to match last year's actual table format
Adds "LCI Strategic Objective Targets" as the primary sheet: four
plain columns (one per objective, no row-label column), each holding
a numbered free-text list of targets, matching the style of last
year's completed version of this table. The previous ratings matrix
is kept as a secondary "Alignment Detail" reference tab.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0187mhodj5WQ6B8rLfzDmXmy
</commit_message>
<xml_diff>
--- a/deliverables/LCI_Funding_Objectives_Matrix.xlsx
+++ b/deliverables/LCI_Funding_Objectives_Matrix.xlsx
@@ -7,10 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LCI Funding x Objectives" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LCI Strategic Targets" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alignment Detail" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'LCI Funding x Objectives'!$A$1:$E$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'LCI Strategic Targets'!$A$1:$D$6</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Alignment Detail'!$A$1:$E$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,8 +82,19 @@
       <color rgb="00444444"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00222222"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00777777"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -113,6 +126,16 @@
         <fgColor rgb="00EBF6F5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7F7F5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -140,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -151,6 +174,15 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -166,9 +198,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -548,6 +577,103 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PARTNERS WORLDWIDE — NIGERIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="26" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>LCI Strategic Objective Targets</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>New funding requests from Homerun Industries, IKORE International and Virtuous Women — October 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="48" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>1.0 Drive A2C (Access 2 Capital) to support entrepreneurs and businesses</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>2.0 Improve A2M (Access 2 Market) for entrepreneurs and businesses</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>3.0 Drive Advocacy + Partnership for Impact</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>4.0 Drive Jobs - Created, sustained</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="220" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>1.1 Raise $50,000 to support Homerun Industries’ rice equipment financing.
+1.2 Raise $50,000 to support Homerun Industries’ cassava backward integration — 200 hectares, including training and input financing.
+1.3 Raise $10,000 to support IKORE’s WINWIN project expansion, providing training and startup kits for women to begin poultry or nutrient-dense crop production from home.
+1.4 Support Virtuous Women’s mechanization services (BSFL) for D’Smiles (amount not specified in the request).
+1.5 Raise $15,000 to support Virtuous Women’s access-to-market micro-loans.</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>2.1 Raise $10,000 to support IKORE’s AgDIL marketplace expansion through its digital leap initiative.</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>No new partnership or LCI-onboarding items were included in the information provided for this cycle.
+Add any advocacy/partnership initiatives (e.g. new LCI onboarding, external partnerships such as last year’s GIZ partnership) you’d like tracked here.</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>No specific jobs-created/sustained targets were included in the information provided for this cycle.
+Add any numeric jobs targets (LCI, number, and date — as in last year’s format) you’d like tracked here.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -580,259 +706,259 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Rating key:</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Direct</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>Indirect</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="10" t="inlineStr">
         <is>
           <t>Minimal</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>Direct = explicit fit · Indirect = plausible but not confirmed by the info given · Minimal = no stated link</t>
         </is>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="9" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Funding Ask</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="4" t="inlineStr">
         <is>
           <t>1.0 Drive A2C (Access 2 Capital) to support entrepreneurs and businesses</t>
         </is>
       </c>
-      <c r="C8" s="10" t="inlineStr">
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>2.0 Improve A2M (Access 2 Market) for entrepreneurs and businesses</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>3.0 Drive Advocacy + Partnership for Impact</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
+      <c r="E8" s="4" t="inlineStr">
         <is>
           <t>4.0 Drive Jobs - Created, sustained</t>
         </is>
       </c>
     </row>
     <row r="9" ht="85" customHeight="1">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>Homerun Industries — Rice equipment financing
 $50,000</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Direct — Equipment financing is itself a capital facility for Homerun to acquire rice-processing equipment.</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="15" t="inlineStr">
         <is>
           <t>Indirect — Added processing capacity can grow throughput for sale, but this ask is capital-focused, not market-linkage-focused.</t>
         </is>
       </c>
-      <c r="D9" s="14" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>Minimal — No advocacy or partnership component stated for this line item.</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>Direct — Processing-line setup and operation typically creates/sustains operational and processing jobs.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="85" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Homerun Industries — Cassava backward integration
 200 ha incl. training &amp; input financing — $50,000</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>Direct — Input financing across 200 hectares is direct capital access for the outgrower farmers involved.</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>Direct — Backward integration secures raw-material supply into Homerun's existing processing/offtake scheme — a direct market-access link for the 200 ha of outgrowers.</t>
         </is>
       </c>
-      <c r="D10" s="14" t="inlineStr">
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>Minimal — No explicit advocacy ask; training delivery may involve partners, but none are named.</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="14" t="inlineStr">
         <is>
           <t>Direct — Training + input financing for 200 ha of outgrowers directly supports farmer livelihoods, building on Homerun's existing 130-farmer outgrower scheme.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="85" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>IKORE International — AgDIL marketplace expansion
 Digital leap — $10,000</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>Minimal — A digital marketplace is not primarily a capital-access tool; any financing effect is indirect at best.</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>Direct — Explicitly a marketplace/market-access expansion for agrifood MSMEs — core to IKORE's market-systems mandate.</t>
         </is>
       </c>
-      <c r="D11" s="14" t="inlineStr">
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>Minimal — No explicit advocacy or partnership detail given for this line item.</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E11" s="15" t="inlineStr">
         <is>
           <t>Indirect — A stronger marketplace can sustain or grow jobs for MSMEs using it, but no direct jobs/training input is stated here.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="85" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>IKORE International — WINWIN project expansion
 Women in FCT — $10,000</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Indirect — Possible capital-access angle if WINWIN includes a financing component, but that isn't specified in the one-line description.</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>Indirect — Plausible market-linkage support for women entrepreneurs, consistent with IKORE's enterprise-support focus, but not confirmed by the description given.</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="15" t="inlineStr">
         <is>
           <t>Indirect — Women's economic-inclusion initiatives often carry an advocacy/partnership dimension; plausible fit, not explicitly confirmed.</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="14" t="inlineStr">
         <is>
           <t>Direct — A women's economic-empowerment project expansion directly supports job creation/sustaining for its women entrepreneur participants.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="85" customHeight="1">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Virtuous Women — Mechanization services (BSFL) for D’Smiles
 Amount not specified in request</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>Minimal — A service/equipment-access ask, not a direct loan or capital product, unless the service itself is financed (not specified).</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C13" s="15" t="inlineStr">
         <is>
           <t>Indirect — Mechanization can improve production efficiency and market readiness, consistent with Virtuous Women's existing tractor-access offering, but no market-linkage detail is stated.</t>
         </is>
       </c>
-      <c r="D13" s="14" t="inlineStr">
+      <c r="D13" s="16" t="inlineStr">
         <is>
           <t>Minimal — No explicit advocacy or partnership detail given for this line item.</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <t>Direct — Mechanization services for a named member group plausibly sustain/expand livelihood activity, consistent with Virtuous Women's existing mechanized-farming access model.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="85" customHeight="1">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="13" t="inlineStr">
         <is>
           <t>Virtuous Women — Access to market micro-loans
 $15,000</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>Direct — Explicitly a micro-loan product — direct capital access.</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>Direct — Explicitly named "access to market" micro-loans — directly supports market access for entrepreneurs.</t>
         </is>
       </c>
-      <c r="D14" s="14" t="inlineStr">
+      <c r="D14" s="16" t="inlineStr">
         <is>
           <t>Minimal — No explicit advocacy or partnership detail given for this line item.</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="14" t="inlineStr">
         <is>
           <t>Direct — Consistent with Virtuous Women's track record (856 entrepreneurs reached via training + loan portfolio), micro-loans sustain member businesses and associated livelihoods.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>Notes:</t>
         </is>
       </c>
     </row>
     <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="15" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>• Ratings are this pack's own assessment of fit, based solely on the one-line descriptions supplied for each ask — not a confirmed classification from Homerun, IKORE or Virtuous Women themselves.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>• “AgDIL”, “WINWIN” and “BSFL” are used exactly as given; none were previously defined in our records, so their full names are not spelled out here. Please confirm if you'd like them expanded.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>• Virtuous Women's mechanization/BSFL ask for D’Smiles did not include a requested amount in the information provided — flagged above rather than estimated.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="15" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>• Objective wording (columns) is reproduced verbatim from the framework supplied.</t>
         </is>

</xml_diff>